<commit_message>
Update equity analysis scripts and output reports
</commit_message>
<xml_diff>
--- a/Equity/output/daily/Backtest_asof_2026-09-29.xlsx
+++ b/Equity/output/daily/Backtest_asof_2026-09-29.xlsx
@@ -415,14 +415,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="20" max="20"/>
+    <col width="31" customWidth="1" min="21" max="21"/>
+    <col width="32" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,17 +470,131 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Setup</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Base Score</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Close asof</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Strategy entry</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Strategy SL</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Strategy T1</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Why</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ADX</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>RVOL</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>ATR%</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>EMA20 dist %</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>vs 20D high %</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>52W high dist %</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Avg value Rs Cr/day</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Alert Entry</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Alert Max high after signal %</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Gain asof close -&gt; best high %</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Alert Result</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Alert Bars held</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Alert Max gain %</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Alert Max drawdown %</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Alert Reached T2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TOURISM FINANCE CORPORATION OF INDIA LIMITED</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
+          <t>TFCILTD</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>30-Sep</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>NO - not in NIFTY500</t>
@@ -466,56 +602,258 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NO DATA (check Yahoo symbol)</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>WOULD BE PICK (rank ~#13, outside top 15) [if it were scanned]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>EMA20 PULLBACK</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>67</v>
+      </c>
+      <c r="G2" t="n">
+        <v>138.9199981689453</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>138.64-139.61</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>132.2653427124023</v>
+      </c>
+      <c r="J2" t="n">
+        <v>148.6443980407715</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Price&gt;EMA20&gt;EMA50&gt;EMA200 | ADX&gt;=25 strong trend | Volume 1.7x avg | OBV rising | BB squeeze before move | Beating NIFTY 1M | Stock hit +7% in 15d 63% of similar setups</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>56.10736089139546</v>
+      </c>
+      <c r="M2" t="n">
+        <v>30.39423649721658</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1.709187851213793</v>
+      </c>
+      <c r="O2" t="n">
+        <v>3.301069145476634</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.2002950972010087</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>-5.912628573259237</v>
+      </c>
+      <c r="R2" t="n">
+        <v>-5.912628573259237</v>
+      </c>
+      <c r="S2" t="n">
+        <v>159.025801833252</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>trigger never hit</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="n">
+        <v>6.896056692575048</v>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TEGA INDUSTRIES LIMITED</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>TEGA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>01-Oct</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NO - not in NIFTY500</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NO DATA (check Yahoo symbol)</t>
+          <t>REJECTED - failed trend/momentum filters</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2060.60009765625</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>RVOL 0.40 &lt; 0.9</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>67.15498194044386</v>
+      </c>
+      <c r="M3" t="n">
+        <v>29.49395764295714</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.4037758872362969</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4.203630186101704</v>
+      </c>
+      <c r="P3" t="n">
+        <v>9.057310138261276</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>-5.259765625000002</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-5.259765625000002</v>
+      </c>
+      <c r="S3" t="n">
+        <v>166.2583813785217</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>trigger never hit</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="n">
+        <v>6.667955732896957</v>
+      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SONA BLW PRECISION FORGINGS LIMITE</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>01-Oct</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NO - not in NIFTY500</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NO DATA (check Yahoo symbol)</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>PICK #10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NEAR BREAKOUT</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>72</v>
+      </c>
+      <c r="G4" t="n">
+        <v>815.6500244140625</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>837.84-849.55</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>803.4817147958967</v>
+      </c>
+      <c r="J4" t="n">
+        <v>902.7547199999999</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Price&gt;EMA20&gt;EMA50&gt;EMA200 | MACD bullish | ADX&gt;=25 strong trend | Volume 2.2x avg | OBV rising | Near 52W high | BB squeeze before move | Beating NIFTY 1M</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>54.99444787147569</v>
+      </c>
+      <c r="M4" t="n">
+        <v>25.12318419076037</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2.158338610634547</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2.739075447693928</v>
+      </c>
+      <c r="P4" t="n">
+        <v>1.442235070371245</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>-2.550773666181305</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-3.359001846675058</v>
+      </c>
+      <c r="S4" t="n">
+        <v>172.9421081451929</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>821.95</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>2.617541218278596</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>STOP HIT</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>1.831010106388065</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>-4.659649276009969</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RANE (MADRAS) LIMITED</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>RML</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>01-Oct</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>NO - not in NIFTY500</t>
@@ -523,18 +861,72 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NO DATA (check Yahoo symbol)</t>
+          <t>REJECTED - no setup pattern</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>1380.900024414062</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>no setup pattern (close 1380.9, 20D high 1440.0, RVOL 0.31, RSI 63) ; RVOL 0.31 &lt; 0.9</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>63.22782231419799</v>
+      </c>
+      <c r="M5" t="n">
+        <v>30.81686402712719</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.3061330847851153</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4.738047157965899</v>
+      </c>
+      <c r="P5" t="n">
+        <v>5.748268918797006</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>-4.104164971245661</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-4.104164971245661</v>
+      </c>
+      <c r="S5" t="n">
+        <v>29.12329694225525</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>trigger never hit</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="n">
+        <v>1.745236813661699</v>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GUJARAT KIDNEY AND SUPER SPECIALITY LIMITED</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>GKSL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>30-Sep</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>NO - not in NIFTY500</t>
@@ -542,18 +934,62 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NO DATA (check Yahoo symbol)</t>
+          <t>REJECTED - short history</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>177.52</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="n">
+        <v>19.27909703779616</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>STOP HIT</t>
+        </is>
+      </c>
+      <c r="X6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>18.18386548129693</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>-0.6421808034089205</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ROLEX RINGS LIMITED</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>ROLEXRINGS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30-Sep</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>NO - not in NIFTY500</t>
@@ -561,10 +997,86 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NO DATA (check Yahoo symbol)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>WOULD BE PICK (rank ~#6, outside top 15) [if it were scanned]</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>MOMENTUM</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>77</v>
+      </c>
+      <c r="G7" t="n">
+        <v>190.5800018310547</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>188.67-192.49</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>178.1923017120361</v>
+      </c>
+      <c r="J7" t="n">
+        <v>203.9206019592285</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Price&gt;EMA20&gt;EMA50&gt;EMA200 | MACD bullish | ADX&gt;=25 strong trend | OBV rising | Near 52W high | BB squeeze before move | Beating NIFTY 1M | Stock hit +7% in 15d 53% of similar setups</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>65.44128478728217</v>
+      </c>
+      <c r="M7" t="n">
+        <v>25.02082621627729</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1.23342758643785</v>
+      </c>
+      <c r="O7" t="n">
+        <v>3.873476909643967</v>
+      </c>
+      <c r="P7" t="n">
+        <v>6.508620502313445</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>-3.965732042434889</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-3.965732042434889</v>
+      </c>
+      <c r="S7" t="n">
+        <v>33.02214787555847</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>192.11</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="n">
+        <v>4.418091136555602</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>open (neither yet)</t>
+        </is>
+      </c>
+      <c r="X7" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>3.586486579437964</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>-2.711991409772785</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -725,7 +1237,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M2" t="n">
         <v>0.2750491159135615</v>
@@ -779,17 +1291,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>open (neither yet)</t>
+          <t>STOP HIT</t>
         </is>
       </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M3" t="n">
         <v>0.5270457697642117</v>
       </c>
       <c r="N3" t="n">
-        <v>-3.700413379854373</v>
+        <v>-5.018027804264912</v>
       </c>
       <c r="O3" t="b">
         <v>0</v>
@@ -887,13 +1399,13 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M5" t="n">
         <v>1.206282970311379</v>
       </c>
       <c r="N5" t="n">
-        <v>-9.379016731910239</v>
+        <v>-12.56245538900785</v>
       </c>
       <c r="O5" t="b">
         <v>0</v>
@@ -945,7 +1457,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" t="n">
         <v>1.461241126051749</v>
@@ -987,7 +1499,7 @@
         <v>1553.178049316406</v>
       </c>
       <c r="H7" t="n">
-        <v>1465.256334863139</v>
+        <v>1465.256334863018</v>
       </c>
       <c r="I7" t="n">
         <v>1645.446052246094</v>
@@ -1003,7 +1515,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" t="n">
         <v>2.925877763328999</v>
@@ -1107,7 +1619,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" t="n">
         <v>6.354977978366194</v>
@@ -1165,7 +1677,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
         <v>0.540839206683863</v>
@@ -1315,7 +1827,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M13" t="n">
         <v>4.193215600510669</v>
@@ -1351,7 +1863,7 @@
         <v>1436.900024414062</v>
       </c>
       <c r="F14" t="n">
-        <v>1420.996848506907</v>
+        <v>1420.996848506902</v>
       </c>
       <c r="G14" t="n">
         <v>1444.084524536133</v>
@@ -1373,13 +1885,13 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M14" t="n">
         <v>3.757167172925291</v>
       </c>
       <c r="N14" t="n">
-        <v>-8.094486585122906</v>
+        <v>-8.481251934353672</v>
       </c>
       <c r="O14" t="b">
         <v>0</v>
@@ -1431,7 +1943,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M15" t="n">
         <v>0.7142857142857117</v>
@@ -1526,14 +2038,26 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>trigger never hit</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+          <t>1743.24</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>open (neither yet)</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>4.690027170647326</v>
+      </c>
+      <c r="N17" t="n">
+        <v>-1.620056658816338</v>
+      </c>
+      <c r="O17" t="b">
+        <v>0</v>
+      </c>
       <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1581,13 +2105,13 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M18" t="n">
         <v>0.5678978440512683</v>
       </c>
       <c r="N18" t="n">
-        <v>-7.518973001116047</v>
+        <v>-9.000049469226257</v>
       </c>
       <c r="O18" t="b">
         <v>0</v>
@@ -1639,7 +2163,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M19" t="n">
         <v>4.395057544322745</v>
@@ -1697,10 +2221,10 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M20" t="n">
-        <v>0.4381037968995694</v>
+        <v>3.229611323298132</v>
       </c>
       <c r="N20" t="n">
         <v>-4.768591327791505</v>
@@ -1739,7 +2263,7 @@
         <v>442.8444876098632</v>
       </c>
       <c r="H21" t="n">
-        <v>426.3956871527336</v>
+        <v>426.3956871305091</v>
       </c>
       <c r="I21" t="n">
         <v>470.5757148339844</v>
@@ -1801,13 +2325,13 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M22" t="n">
         <v>2.306607953648143</v>
       </c>
       <c r="N22" t="n">
-        <v>-6.794286618915645</v>
+        <v>-11.29766222801022</v>
       </c>
       <c r="O22" t="b">
         <v>0</v>
@@ -1859,7 +2383,7 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M23" t="n">
         <v>0.05789778409390767</v>
@@ -1917,7 +2441,7 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
         <v>0.6974422686433668</v>
@@ -1975,13 +2499,13 @@
         </is>
       </c>
       <c r="L25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M25" t="n">
         <v>1.960784313725483</v>
       </c>
       <c r="N25" t="n">
-        <v>-6.107267843948239</v>
+        <v>-7.727797001153403</v>
       </c>
       <c r="O25" t="b">
         <v>0</v>
@@ -2033,7 +2557,7 @@
         </is>
       </c>
       <c r="L26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M26" t="n">
         <v>2.009205887415622</v>

</xml_diff>